<commit_message>
feat(ot): expand probetas capacity dynamically beyond 12 items, auto-normalize -26 suffix, and update OT-0000-Geofal.xlsx
</commit_message>
<xml_diff>
--- a/app/templates/OT/OT-CONCRETO/OT-0000-Geofal.xlsx
+++ b/app/templates/OT/OT-CONCRETO/OT-0000-Geofal.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Equipo\Desktop\miguel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\OT\OT-CONCRETO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70C8BF50-0BDA-4285-A549-894A23D87A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{323A4CD5-00F4-4932-A24D-B5EFAC25307F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -352,9 +352,6 @@
     <t>ITEM</t>
   </si>
   <si>
-    <t>OT DESIGADA A:                                                                       (Colocar el nombre de los técnicos)</t>
-  </si>
-  <si>
     <t>F-LEM-P-02.02</t>
   </si>
   <si>
@@ -383,6 +380,9 @@
   </si>
   <si>
     <t>Resistencia a la Flexión del concreto en vigas NTP 339.078/079</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT DESIGADA A:                                                                  </t>
   </si>
 </sst>
 </file>
@@ -398,8 +398,8 @@
     <numFmt numFmtId="169" formatCode="000&quot;-AG-24&quot;"/>
     <numFmt numFmtId="170" formatCode="000&quot;-CO-24&quot;"/>
     <numFmt numFmtId="171" formatCode="000&quot;-SU-23&quot;"/>
-    <numFmt numFmtId="174" formatCode="000\-&quot;26-LEM&quot;"/>
-    <numFmt numFmtId="175" formatCode="000\-&quot;26&quot;"/>
+    <numFmt numFmtId="172" formatCode="000\-&quot;26-LEM&quot;"/>
+    <numFmt numFmtId="173" formatCode="000\-&quot;26&quot;"/>
   </numFmts>
   <fonts count="17" x14ac:knownFonts="1">
     <font>
@@ -718,7 +718,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -783,20 +783,78 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="175" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="174" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -810,80 +868,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="6" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="171" fontId="6" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="171" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -892,6 +881,90 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="168" fontId="6" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="6" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -901,29 +974,38 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -942,9 +1024,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -958,7 +1037,7 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -973,93 +1052,8 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1395,9 +1389,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1435,9 +1429,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1470,26 +1464,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1522,26 +1499,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1738,16 +1698,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="48"/>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="58" t="s">
+      <c r="A1" s="49"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
       <c r="I1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1756,14 +1716,14 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
+      <c r="A2" s="49"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
       <c r="I2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1772,14 +1732,14 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="48"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
+      <c r="A3" s="49"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
       <c r="I3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1788,14 +1748,14 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="48"/>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
+      <c r="A4" s="49"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
       <c r="I4" s="1" t="s">
         <v>5</v>
       </c>
@@ -1820,10 +1780,10 @@
       <c r="A6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="56">
+      <c r="B6" s="47">
         <v>716</v>
       </c>
-      <c r="C6" s="56"/>
+      <c r="C6" s="47"/>
       <c r="D6" s="16"/>
       <c r="E6" s="15"/>
       <c r="F6" s="15" t="s">
@@ -1849,10 +1809,10 @@
       <c r="F7" s="15"/>
       <c r="G7" s="15"/>
       <c r="H7" s="16"/>
-      <c r="I7" s="57" t="s">
+      <c r="I7" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="57"/>
+      <c r="J7" s="48"/>
     </row>
     <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14"/>
@@ -1870,18 +1830,18 @@
       <c r="A9" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="77" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28" t="s">
+      <c r="C9" s="77"/>
+      <c r="D9" s="77"/>
+      <c r="E9" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
+      <c r="F9" s="77"/>
+      <c r="G9" s="77"/>
+      <c r="H9" s="77"/>
+      <c r="I9" s="77"/>
       <c r="J9" s="13" t="s">
         <v>15</v>
       </c>
@@ -1890,287 +1850,287 @@
       <c r="A10" s="12">
         <v>1</v>
       </c>
-      <c r="B10" s="36">
+      <c r="B10" s="78">
         <v>2547</v>
       </c>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="38" t="s">
+      <c r="C10" s="79"/>
+      <c r="D10" s="79"/>
+      <c r="E10" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="40"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="62"/>
       <c r="J10" s="22">
         <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="33"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="55"/>
+      <c r="E11" s="51"/>
+      <c r="F11" s="52"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="52"/>
+      <c r="I11" s="53"/>
       <c r="J11" s="12"/>
     </row>
     <row r="12" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12"/>
-      <c r="B12" s="36">
+      <c r="B12" s="78">
         <v>2570</v>
       </c>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="44"/>
-      <c r="I12" s="44"/>
+      <c r="C12" s="79"/>
+      <c r="D12" s="79"/>
+      <c r="E12" s="75"/>
+      <c r="F12" s="76"/>
+      <c r="G12" s="76"/>
+      <c r="H12" s="76"/>
+      <c r="I12" s="76"/>
       <c r="J12" s="12"/>
     </row>
     <row r="13" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12"/>
-      <c r="B13" s="34"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="31"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="33"/>
+      <c r="B13" s="73"/>
+      <c r="C13" s="74"/>
+      <c r="D13" s="74"/>
+      <c r="E13" s="51"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="52"/>
+      <c r="I13" s="53"/>
       <c r="J13" s="12"/>
     </row>
     <row r="14" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12"/>
-      <c r="B14" s="41"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="32"/>
-      <c r="I14" s="33"/>
+      <c r="B14" s="54"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="51"/>
+      <c r="F14" s="52"/>
+      <c r="G14" s="52"/>
+      <c r="H14" s="52"/>
+      <c r="I14" s="53"/>
       <c r="J14" s="12"/>
     </row>
     <row r="15" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12"/>
-      <c r="B15" s="45"/>
-      <c r="C15" s="39"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39"/>
-      <c r="H15" s="39"/>
-      <c r="I15" s="40"/>
+      <c r="B15" s="72"/>
+      <c r="C15" s="61"/>
+      <c r="D15" s="62"/>
+      <c r="E15" s="60"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="61"/>
+      <c r="H15" s="61"/>
+      <c r="I15" s="62"/>
       <c r="J15" s="22"/>
     </row>
     <row r="16" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="12"/>
-      <c r="B16" s="34"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="32"/>
-      <c r="I16" s="33"/>
+      <c r="B16" s="73"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="51"/>
+      <c r="F16" s="52"/>
+      <c r="G16" s="52"/>
+      <c r="H16" s="52"/>
+      <c r="I16" s="53"/>
       <c r="J16" s="12"/>
     </row>
     <row r="17" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12"/>
-      <c r="B17" s="41"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="32"/>
-      <c r="H17" s="32"/>
-      <c r="I17" s="33"/>
+      <c r="B17" s="54"/>
+      <c r="C17" s="55"/>
+      <c r="D17" s="55"/>
+      <c r="E17" s="51"/>
+      <c r="F17" s="52"/>
+      <c r="G17" s="52"/>
+      <c r="H17" s="52"/>
+      <c r="I17" s="53"/>
       <c r="J17" s="12"/>
     </row>
     <row r="18" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="40"/>
+      <c r="B18" s="58"/>
+      <c r="C18" s="59"/>
+      <c r="D18" s="59"/>
+      <c r="E18" s="60"/>
+      <c r="F18" s="61"/>
+      <c r="G18" s="61"/>
+      <c r="H18" s="61"/>
+      <c r="I18" s="62"/>
       <c r="J18" s="22"/>
     </row>
     <row r="19" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12"/>
-      <c r="B19" s="29"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="32"/>
-      <c r="I19" s="33"/>
+      <c r="B19" s="58"/>
+      <c r="C19" s="59"/>
+      <c r="D19" s="59"/>
+      <c r="E19" s="51"/>
+      <c r="F19" s="52"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="52"/>
+      <c r="I19" s="53"/>
       <c r="J19" s="12"/>
     </row>
     <row r="20" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="12"/>
-      <c r="B20" s="41"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="43"/>
-      <c r="F20" s="44"/>
-      <c r="G20" s="44"/>
-      <c r="H20" s="44"/>
-      <c r="I20" s="44"/>
+      <c r="B20" s="54"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="75"/>
+      <c r="F20" s="76"/>
+      <c r="G20" s="76"/>
+      <c r="H20" s="76"/>
+      <c r="I20" s="76"/>
       <c r="J20" s="12"/>
     </row>
     <row r="21" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="32"/>
-      <c r="I21" s="33"/>
+      <c r="B21" s="58"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="51"/>
+      <c r="F21" s="52"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="52"/>
+      <c r="I21" s="53"/>
       <c r="J21" s="12"/>
     </row>
     <row r="22" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12"/>
-      <c r="B22" s="34"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="32"/>
-      <c r="H22" s="32"/>
-      <c r="I22" s="33"/>
+      <c r="B22" s="73"/>
+      <c r="C22" s="74"/>
+      <c r="D22" s="74"/>
+      <c r="E22" s="51"/>
+      <c r="F22" s="52"/>
+      <c r="G22" s="52"/>
+      <c r="H22" s="52"/>
+      <c r="I22" s="53"/>
       <c r="J22" s="12"/>
     </row>
     <row r="23" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="12"/>
-      <c r="B23" s="41"/>
-      <c r="C23" s="42"/>
-      <c r="D23" s="42"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="32"/>
-      <c r="G23" s="32"/>
-      <c r="H23" s="32"/>
-      <c r="I23" s="33"/>
+      <c r="B23" s="54"/>
+      <c r="C23" s="55"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="51"/>
+      <c r="F23" s="52"/>
+      <c r="G23" s="52"/>
+      <c r="H23" s="52"/>
+      <c r="I23" s="53"/>
       <c r="J23" s="12"/>
     </row>
     <row r="24" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
-      <c r="B24" s="48"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="33"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="51"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="52"/>
+      <c r="H24" s="52"/>
+      <c r="I24" s="53"/>
       <c r="J24" s="12"/>
     </row>
     <row r="25" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12"/>
-      <c r="B25" s="41"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="48"/>
-      <c r="H25" s="48"/>
-      <c r="I25" s="48"/>
+      <c r="B25" s="54"/>
+      <c r="C25" s="55"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="57"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="49"/>
       <c r="J25" s="12"/>
     </row>
     <row r="26" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="12"/>
-      <c r="B26" s="41"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="33"/>
+      <c r="B26" s="54"/>
+      <c r="C26" s="55"/>
+      <c r="D26" s="55"/>
+      <c r="E26" s="56"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="52"/>
+      <c r="I26" s="53"/>
       <c r="J26" s="12"/>
     </row>
     <row r="27" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="12"/>
-      <c r="B27" s="48"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
-      <c r="I27" s="48"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="49"/>
+      <c r="D27" s="49"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="49"/>
+      <c r="H27" s="49"/>
+      <c r="I27" s="49"/>
       <c r="J27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="12"/>
-      <c r="B28" s="48"/>
-      <c r="C28" s="48"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="33"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="52"/>
+      <c r="H28" s="52"/>
+      <c r="I28" s="53"/>
       <c r="J28" s="12"/>
     </row>
     <row r="29" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="12"/>
-      <c r="B29" s="48"/>
-      <c r="C29" s="48"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="40"/>
+      <c r="B29" s="49"/>
+      <c r="C29" s="49"/>
+      <c r="D29" s="49"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="61"/>
+      <c r="G29" s="61"/>
+      <c r="H29" s="61"/>
+      <c r="I29" s="62"/>
       <c r="J29" s="22"/>
     </row>
     <row r="30" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="12"/>
-      <c r="B30" s="48"/>
-      <c r="C30" s="48"/>
-      <c r="D30" s="48"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
-      <c r="I30" s="33"/>
+      <c r="B30" s="49"/>
+      <c r="C30" s="49"/>
+      <c r="D30" s="49"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="52"/>
+      <c r="H30" s="52"/>
+      <c r="I30" s="53"/>
       <c r="J30" s="12"/>
     </row>
     <row r="31" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="12"/>
-      <c r="B31" s="48"/>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="48"/>
-      <c r="H31" s="48"/>
-      <c r="I31" s="48"/>
+      <c r="B31" s="49"/>
+      <c r="C31" s="49"/>
+      <c r="D31" s="49"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="49"/>
+      <c r="G31" s="49"/>
+      <c r="H31" s="49"/>
+      <c r="I31" s="49"/>
       <c r="J31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="55" t="s">
+      <c r="A32" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="B32" s="55"/>
-      <c r="C32" s="51">
+      <c r="B32" s="64"/>
+      <c r="C32" s="69">
         <v>45524</v>
       </c>
-      <c r="D32" s="52"/>
+      <c r="D32" s="70"/>
       <c r="E32" s="5" t="s">
         <v>19</v>
       </c>
@@ -2187,15 +2147,15 @@
       <c r="J32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="55" t="s">
+      <c r="A33" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="55"/>
-      <c r="C33" s="53">
+      <c r="B33" s="64"/>
+      <c r="C33" s="71">
         <f>+F33-F32+1</f>
         <v>14</v>
       </c>
-      <c r="D33" s="53"/>
+      <c r="D33" s="71"/>
       <c r="E33" s="5" t="s">
         <v>23</v>
       </c>
@@ -2212,88 +2172,88 @@
       <c r="J33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="54" t="s">
+      <c r="A34" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B34" s="54"/>
-      <c r="C34" s="54"/>
-      <c r="D34" s="54"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="54"/>
-      <c r="G34" s="54"/>
-      <c r="H34" s="54"/>
-      <c r="I34" s="54"/>
-      <c r="J34" s="54"/>
+      <c r="B34" s="63"/>
+      <c r="C34" s="63"/>
+      <c r="D34" s="63"/>
+      <c r="E34" s="63"/>
+      <c r="F34" s="63"/>
+      <c r="G34" s="63"/>
+      <c r="H34" s="63"/>
+      <c r="I34" s="63"/>
+      <c r="J34" s="63"/>
     </row>
     <row r="35" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="46" t="s">
+      <c r="A35" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="B35" s="46"/>
-      <c r="C35" s="46"/>
-      <c r="D35" s="46"/>
-      <c r="E35" s="46"/>
-      <c r="F35" s="46"/>
-      <c r="G35" s="46"/>
-      <c r="H35" s="46"/>
-      <c r="I35" s="46"/>
-      <c r="J35" s="46"/>
+      <c r="B35" s="65"/>
+      <c r="C35" s="65"/>
+      <c r="D35" s="65"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="65"/>
+      <c r="G35" s="65"/>
+      <c r="H35" s="65"/>
+      <c r="I35" s="65"/>
+      <c r="J35" s="65"/>
     </row>
     <row r="36" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="46"/>
-      <c r="B36" s="46"/>
-      <c r="C36" s="46"/>
-      <c r="D36" s="46"/>
-      <c r="E36" s="46"/>
-      <c r="F36" s="46"/>
-      <c r="G36" s="46"/>
-      <c r="H36" s="46"/>
-      <c r="I36" s="46"/>
-      <c r="J36" s="46"/>
+      <c r="A36" s="65"/>
+      <c r="B36" s="65"/>
+      <c r="C36" s="65"/>
+      <c r="D36" s="65"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="65"/>
+      <c r="G36" s="65"/>
+      <c r="H36" s="65"/>
+      <c r="I36" s="65"/>
+      <c r="J36" s="65"/>
     </row>
     <row r="37" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="46"/>
-      <c r="B37" s="46"/>
-      <c r="C37" s="46"/>
-      <c r="D37" s="46"/>
-      <c r="E37" s="46"/>
-      <c r="F37" s="46"/>
-      <c r="G37" s="46"/>
-      <c r="H37" s="46"/>
-      <c r="I37" s="46"/>
-      <c r="J37" s="46"/>
+      <c r="A37" s="65"/>
+      <c r="B37" s="65"/>
+      <c r="C37" s="65"/>
+      <c r="D37" s="65"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="65"/>
+      <c r="H37" s="65"/>
+      <c r="I37" s="65"/>
+      <c r="J37" s="65"/>
     </row>
     <row r="38" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="46"/>
-      <c r="B38" s="46"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="46"/>
-      <c r="F38" s="46"/>
-      <c r="G38" s="46"/>
-      <c r="H38" s="46"/>
-      <c r="I38" s="46"/>
-      <c r="J38" s="46"/>
+      <c r="A38" s="65"/>
+      <c r="B38" s="65"/>
+      <c r="C38" s="65"/>
+      <c r="D38" s="65"/>
+      <c r="E38" s="65"/>
+      <c r="F38" s="65"/>
+      <c r="G38" s="65"/>
+      <c r="H38" s="65"/>
+      <c r="I38" s="65"/>
+      <c r="J38" s="65"/>
     </row>
     <row r="39" spans="1:10" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="49" t="s">
+      <c r="A39" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="B39" s="50"/>
-      <c r="C39" s="45" t="s">
+      <c r="B39" s="68"/>
+      <c r="C39" s="72" t="s">
         <v>29</v>
       </c>
-      <c r="D39" s="39"/>
-      <c r="E39" s="39"/>
-      <c r="F39" s="40"/>
+      <c r="D39" s="61"/>
+      <c r="E39" s="61"/>
+      <c r="F39" s="62"/>
       <c r="G39" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="H39" s="47" t="s">
+      <c r="H39" s="66" t="s">
         <v>31</v>
       </c>
-      <c r="I39" s="48"/>
-      <c r="J39" s="48"/>
+      <c r="I39" s="49"/>
+      <c r="J39" s="49"/>
     </row>
     <row r="46" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -2301,6 +2261,49 @@
     </row>
   </sheetData>
   <mergeCells count="59">
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="E9:I9"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E19:I19"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:I13"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:I10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="E11:I11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="E12:I12"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E15:I15"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E22:I22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E14:I14"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="E16:I16"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="E20:I20"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="E18:I18"/>
+    <mergeCell ref="A35:J38"/>
+    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C39:F39"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="A34:J34"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="B31:D31"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="I7:J7"/>
     <mergeCell ref="B28:D28"/>
@@ -2317,49 +2320,6 @@
     <mergeCell ref="E25:I25"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="E21:I21"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="E29:I29"/>
-    <mergeCell ref="A34:J34"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="A35:J38"/>
-    <mergeCell ref="H39:J39"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C39:F39"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="E22:I22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="E14:I14"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="E16:I16"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="E20:I20"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="E18:I18"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="E9:I9"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E19:I19"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:I13"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:I10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="E11:I11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="E12:I12"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="E15:I15"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.59055118110236227" right="0.39370078740157483" top="0.78740157480314965" bottom="0.39370078740157483" header="0" footer="0"/>
@@ -2394,16 +2354,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="48"/>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="58" t="s">
+      <c r="A1" s="49"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
       <c r="I1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2412,14 +2372,14 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
+      <c r="A2" s="49"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
       <c r="I2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2428,14 +2388,14 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="48"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
+      <c r="A3" s="49"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
       <c r="I3" s="1" t="s">
         <v>4</v>
       </c>
@@ -2444,14 +2404,14 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="48"/>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
+      <c r="A4" s="49"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
       <c r="I4" s="1" t="s">
         <v>5</v>
       </c>
@@ -2476,10 +2436,10 @@
       <c r="A6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="56">
+      <c r="B6" s="47">
         <v>839</v>
       </c>
-      <c r="C6" s="56"/>
+      <c r="C6" s="47"/>
       <c r="D6" s="16"/>
       <c r="E6" s="15"/>
       <c r="F6" s="15" t="s">
@@ -2505,10 +2465,10 @@
       <c r="F7" s="15"/>
       <c r="G7" s="15"/>
       <c r="H7" s="16"/>
-      <c r="I7" s="57" t="s">
+      <c r="I7" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="57"/>
+      <c r="J7" s="48"/>
     </row>
     <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14"/>
@@ -2526,18 +2486,18 @@
       <c r="A9" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="77" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28" t="s">
+      <c r="C9" s="77"/>
+      <c r="D9" s="77"/>
+      <c r="E9" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
+      <c r="F9" s="77"/>
+      <c r="G9" s="77"/>
+      <c r="H9" s="77"/>
+      <c r="I9" s="77"/>
       <c r="J9" s="13" t="s">
         <v>15</v>
       </c>
@@ -2546,199 +2506,199 @@
       <c r="A10" s="12">
         <v>1</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="64" t="s">
+      <c r="C10" s="74"/>
+      <c r="D10" s="74"/>
+      <c r="E10" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="68"/>
-      <c r="G10" s="68"/>
-      <c r="H10" s="68"/>
-      <c r="I10" s="69"/>
+      <c r="F10" s="81"/>
+      <c r="G10" s="81"/>
+      <c r="H10" s="81"/>
+      <c r="I10" s="82"/>
       <c r="J10" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
-      <c r="B11" s="41"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="31" t="s">
+      <c r="B11" s="54"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="55"/>
+      <c r="E11" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="33"/>
+      <c r="F11" s="52"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="52"/>
+      <c r="I11" s="53"/>
       <c r="J11" s="12">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12"/>
-      <c r="B12" s="36"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="64" t="s">
+      <c r="B12" s="78"/>
+      <c r="C12" s="79"/>
+      <c r="D12" s="79"/>
+      <c r="E12" s="83" t="s">
         <v>35</v>
       </c>
-      <c r="F12" s="65"/>
-      <c r="G12" s="65"/>
-      <c r="H12" s="65"/>
-      <c r="I12" s="66"/>
+      <c r="F12" s="84"/>
+      <c r="G12" s="84"/>
+      <c r="H12" s="84"/>
+      <c r="I12" s="85"/>
       <c r="J12" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12"/>
-      <c r="B13" s="48"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="31" t="s">
+      <c r="B13" s="49"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="33"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="52"/>
+      <c r="I13" s="53"/>
       <c r="J13" s="12">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12"/>
-      <c r="B14" s="34"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="45" t="s">
+      <c r="B14" s="73"/>
+      <c r="C14" s="74"/>
+      <c r="D14" s="74"/>
+      <c r="E14" s="72" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="39"/>
-      <c r="I14" s="40"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="61"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="62"/>
       <c r="J14" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="70" t="s">
+      <c r="B15" s="73"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="80" t="s">
         <v>38</v>
       </c>
-      <c r="F15" s="68"/>
-      <c r="G15" s="68"/>
-      <c r="H15" s="68"/>
-      <c r="I15" s="69"/>
+      <c r="F15" s="81"/>
+      <c r="G15" s="81"/>
+      <c r="H15" s="81"/>
+      <c r="I15" s="82"/>
       <c r="J15" s="12">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="12"/>
-      <c r="B16" s="45"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="61" t="s">
+      <c r="B16" s="72"/>
+      <c r="C16" s="61"/>
+      <c r="D16" s="62"/>
+      <c r="E16" s="86" t="s">
         <v>39</v>
       </c>
-      <c r="F16" s="62"/>
-      <c r="G16" s="62"/>
-      <c r="H16" s="62"/>
-      <c r="I16" s="63"/>
+      <c r="F16" s="87"/>
+      <c r="G16" s="87"/>
+      <c r="H16" s="87"/>
+      <c r="I16" s="88"/>
       <c r="J16" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12"/>
-      <c r="B17" s="45"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="64" t="s">
+      <c r="B17" s="72"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="62"/>
+      <c r="E17" s="83" t="s">
         <v>40</v>
       </c>
-      <c r="F17" s="65"/>
-      <c r="G17" s="65"/>
-      <c r="H17" s="65"/>
-      <c r="I17" s="66"/>
+      <c r="F17" s="84"/>
+      <c r="G17" s="84"/>
+      <c r="H17" s="84"/>
+      <c r="I17" s="85"/>
       <c r="J17" s="12">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12"/>
-      <c r="B18" s="48"/>
-      <c r="C18" s="48"/>
-      <c r="D18" s="48"/>
-      <c r="E18" s="67" t="s">
+      <c r="B18" s="49"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="89" t="s">
         <v>41</v>
       </c>
-      <c r="F18" s="68"/>
-      <c r="G18" s="68"/>
-      <c r="H18" s="68"/>
-      <c r="I18" s="69"/>
+      <c r="F18" s="81"/>
+      <c r="G18" s="81"/>
+      <c r="H18" s="81"/>
+      <c r="I18" s="82"/>
       <c r="J18" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12"/>
-      <c r="B19" s="29"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="31" t="s">
+      <c r="B19" s="58"/>
+      <c r="C19" s="59"/>
+      <c r="D19" s="59"/>
+      <c r="E19" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="32"/>
-      <c r="I19" s="33"/>
+      <c r="F19" s="52"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="52"/>
+      <c r="I19" s="53"/>
       <c r="J19" s="12">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="12"/>
-      <c r="B20" s="41"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="38" t="s">
+      <c r="B20" s="54"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="60" t="s">
         <v>43</v>
       </c>
-      <c r="F20" s="39"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="39"/>
-      <c r="I20" s="40"/>
+      <c r="F20" s="61"/>
+      <c r="G20" s="61"/>
+      <c r="H20" s="61"/>
+      <c r="I20" s="62"/>
       <c r="J20" s="12">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="48"/>
-      <c r="G21" s="48"/>
-      <c r="H21" s="48"/>
-      <c r="I21" s="48"/>
+      <c r="B21" s="58"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="57"/>
+      <c r="F21" s="49"/>
+      <c r="G21" s="49"/>
+      <c r="H21" s="49"/>
+      <c r="I21" s="49"/>
       <c r="J21" s="12"/>
     </row>
     <row r="22" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12"/>
-      <c r="B22" s="34"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
+      <c r="B22" s="73"/>
+      <c r="C22" s="74"/>
+      <c r="D22" s="74"/>
       <c r="E22" s="23"/>
       <c r="F22" s="24"/>
       <c r="G22" s="24"/>
@@ -2748,116 +2708,116 @@
     </row>
     <row r="23" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="12"/>
-      <c r="B23" s="41"/>
-      <c r="C23" s="42"/>
-      <c r="D23" s="42"/>
+      <c r="B23" s="54"/>
+      <c r="C23" s="55"/>
+      <c r="D23" s="55"/>
       <c r="J23" s="12"/>
     </row>
     <row r="24" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
-      <c r="B24" s="48"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="33"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="51"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="52"/>
+      <c r="H24" s="52"/>
+      <c r="I24" s="53"/>
       <c r="J24" s="12"/>
     </row>
     <row r="25" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12"/>
-      <c r="B25" s="41"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="48"/>
-      <c r="H25" s="48"/>
-      <c r="I25" s="48"/>
+      <c r="B25" s="54"/>
+      <c r="C25" s="55"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="57"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="49"/>
       <c r="J25" s="12"/>
     </row>
     <row r="26" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="12"/>
-      <c r="B26" s="41"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="33"/>
+      <c r="B26" s="54"/>
+      <c r="C26" s="55"/>
+      <c r="D26" s="55"/>
+      <c r="E26" s="56"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="52"/>
+      <c r="I26" s="53"/>
       <c r="J26" s="12"/>
     </row>
     <row r="27" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="12"/>
-      <c r="B27" s="48"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
-      <c r="I27" s="48"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="49"/>
+      <c r="D27" s="49"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="49"/>
+      <c r="H27" s="49"/>
+      <c r="I27" s="49"/>
       <c r="J27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="12"/>
-      <c r="B28" s="48"/>
-      <c r="C28" s="48"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="33"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="52"/>
+      <c r="H28" s="52"/>
+      <c r="I28" s="53"/>
       <c r="J28" s="12"/>
     </row>
     <row r="29" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="12"/>
-      <c r="B29" s="48"/>
-      <c r="C29" s="48"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="40"/>
+      <c r="B29" s="49"/>
+      <c r="C29" s="49"/>
+      <c r="D29" s="49"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="61"/>
+      <c r="G29" s="61"/>
+      <c r="H29" s="61"/>
+      <c r="I29" s="62"/>
       <c r="J29" s="22"/>
     </row>
     <row r="30" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="12"/>
-      <c r="B30" s="48"/>
-      <c r="C30" s="48"/>
-      <c r="D30" s="48"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
-      <c r="I30" s="33"/>
+      <c r="B30" s="49"/>
+      <c r="C30" s="49"/>
+      <c r="D30" s="49"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="52"/>
+      <c r="H30" s="52"/>
+      <c r="I30" s="53"/>
       <c r="J30" s="12"/>
     </row>
     <row r="31" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="12"/>
-      <c r="B31" s="48"/>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="48"/>
-      <c r="H31" s="48"/>
-      <c r="I31" s="48"/>
+      <c r="B31" s="49"/>
+      <c r="C31" s="49"/>
+      <c r="D31" s="49"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="49"/>
+      <c r="G31" s="49"/>
+      <c r="H31" s="49"/>
+      <c r="I31" s="49"/>
       <c r="J31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="55" t="s">
+      <c r="A32" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="B32" s="55"/>
-      <c r="C32" s="51">
+      <c r="B32" s="64"/>
+      <c r="C32" s="69">
         <v>45555</v>
       </c>
-      <c r="D32" s="52"/>
+      <c r="D32" s="70"/>
       <c r="E32" s="5" t="s">
         <v>19</v>
       </c>
@@ -2874,15 +2834,15 @@
       <c r="J32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="55" t="s">
+      <c r="A33" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="55"/>
-      <c r="C33" s="53">
+      <c r="B33" s="64"/>
+      <c r="C33" s="71">
         <f>+F33-F32+1</f>
         <v>5</v>
       </c>
-      <c r="D33" s="53"/>
+      <c r="D33" s="71"/>
       <c r="E33" s="5" t="s">
         <v>23</v>
       </c>
@@ -2899,88 +2859,88 @@
       <c r="J33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="54" t="s">
+      <c r="A34" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B34" s="54"/>
-      <c r="C34" s="54"/>
-      <c r="D34" s="54"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="54"/>
-      <c r="G34" s="54"/>
-      <c r="H34" s="54"/>
-      <c r="I34" s="54"/>
-      <c r="J34" s="54"/>
+      <c r="B34" s="63"/>
+      <c r="C34" s="63"/>
+      <c r="D34" s="63"/>
+      <c r="E34" s="63"/>
+      <c r="F34" s="63"/>
+      <c r="G34" s="63"/>
+      <c r="H34" s="63"/>
+      <c r="I34" s="63"/>
+      <c r="J34" s="63"/>
     </row>
     <row r="35" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="46" t="s">
+      <c r="A35" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="B35" s="46"/>
-      <c r="C35" s="46"/>
-      <c r="D35" s="46"/>
-      <c r="E35" s="46"/>
-      <c r="F35" s="46"/>
-      <c r="G35" s="46"/>
-      <c r="H35" s="46"/>
-      <c r="I35" s="46"/>
-      <c r="J35" s="46"/>
+      <c r="B35" s="65"/>
+      <c r="C35" s="65"/>
+      <c r="D35" s="65"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="65"/>
+      <c r="G35" s="65"/>
+      <c r="H35" s="65"/>
+      <c r="I35" s="65"/>
+      <c r="J35" s="65"/>
     </row>
     <row r="36" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="46"/>
-      <c r="B36" s="46"/>
-      <c r="C36" s="46"/>
-      <c r="D36" s="46"/>
-      <c r="E36" s="46"/>
-      <c r="F36" s="46"/>
-      <c r="G36" s="46"/>
-      <c r="H36" s="46"/>
-      <c r="I36" s="46"/>
-      <c r="J36" s="46"/>
+      <c r="A36" s="65"/>
+      <c r="B36" s="65"/>
+      <c r="C36" s="65"/>
+      <c r="D36" s="65"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="65"/>
+      <c r="G36" s="65"/>
+      <c r="H36" s="65"/>
+      <c r="I36" s="65"/>
+      <c r="J36" s="65"/>
     </row>
     <row r="37" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="46"/>
-      <c r="B37" s="46"/>
-      <c r="C37" s="46"/>
-      <c r="D37" s="46"/>
-      <c r="E37" s="46"/>
-      <c r="F37" s="46"/>
-      <c r="G37" s="46"/>
-      <c r="H37" s="46"/>
-      <c r="I37" s="46"/>
-      <c r="J37" s="46"/>
+      <c r="A37" s="65"/>
+      <c r="B37" s="65"/>
+      <c r="C37" s="65"/>
+      <c r="D37" s="65"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="65"/>
+      <c r="H37" s="65"/>
+      <c r="I37" s="65"/>
+      <c r="J37" s="65"/>
     </row>
     <row r="38" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="46"/>
-      <c r="B38" s="46"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="46"/>
-      <c r="F38" s="46"/>
-      <c r="G38" s="46"/>
-      <c r="H38" s="46"/>
-      <c r="I38" s="46"/>
-      <c r="J38" s="46"/>
+      <c r="A38" s="65"/>
+      <c r="B38" s="65"/>
+      <c r="C38" s="65"/>
+      <c r="D38" s="65"/>
+      <c r="E38" s="65"/>
+      <c r="F38" s="65"/>
+      <c r="G38" s="65"/>
+      <c r="H38" s="65"/>
+      <c r="I38" s="65"/>
+      <c r="J38" s="65"/>
     </row>
     <row r="39" spans="1:10" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="49" t="s">
+      <c r="A39" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="B39" s="50"/>
-      <c r="C39" s="45" t="s">
+      <c r="B39" s="68"/>
+      <c r="C39" s="72" t="s">
         <v>29</v>
       </c>
-      <c r="D39" s="39"/>
-      <c r="E39" s="39"/>
-      <c r="F39" s="40"/>
+      <c r="D39" s="61"/>
+      <c r="E39" s="61"/>
+      <c r="F39" s="62"/>
       <c r="G39" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="H39" s="47" t="s">
+      <c r="H39" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="I39" s="48"/>
-      <c r="J39" s="48"/>
+      <c r="I39" s="49"/>
+      <c r="J39" s="49"/>
     </row>
     <row r="46" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -2988,6 +2948,47 @@
     </row>
   </sheetData>
   <mergeCells count="57">
+    <mergeCell ref="E16:I16"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="E18:I18"/>
+    <mergeCell ref="E19:I19"/>
+    <mergeCell ref="A34:J34"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E20:I20"/>
+    <mergeCell ref="E21:I21"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="C39:F39"/>
+    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="A35:J38"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
     <mergeCell ref="E13:I13"/>
     <mergeCell ref="E14:I14"/>
     <mergeCell ref="E15:I15"/>
@@ -3004,47 +3005,6 @@
     <mergeCell ref="E10:I10"/>
     <mergeCell ref="E11:I11"/>
     <mergeCell ref="E12:I12"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C39:F39"/>
-    <mergeCell ref="H39:J39"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="A35:J38"/>
-    <mergeCell ref="E16:I16"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="E18:I18"/>
-    <mergeCell ref="E19:I19"/>
-    <mergeCell ref="A34:J34"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="E28:I28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="E29:I29"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E20:I20"/>
-    <mergeCell ref="E21:I21"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="E25:I25"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.59055118110236227" right="0.39370078740157483" top="0.78740157480314965" bottom="0.39370078740157483" header="0" footer="0"/>
@@ -3076,70 +3036,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72"/>
-      <c r="B1" s="73"/>
-      <c r="C1" s="79" t="s">
+      <c r="A1" s="100"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="106" t="s">
         <v>62</v>
       </c>
-      <c r="D1" s="80"/>
-      <c r="E1" s="80"/>
-      <c r="F1" s="80"/>
-      <c r="G1" s="80"/>
-      <c r="H1" s="81"/>
+      <c r="D1" s="107"/>
+      <c r="E1" s="107"/>
+      <c r="F1" s="107"/>
+      <c r="G1" s="107"/>
+      <c r="H1" s="108"/>
       <c r="I1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="74"/>
-      <c r="B2" s="75"/>
-      <c r="C2" s="82"/>
-      <c r="D2" s="83"/>
-      <c r="E2" s="83"/>
-      <c r="F2" s="83"/>
-      <c r="G2" s="83"/>
-      <c r="H2" s="84"/>
+      <c r="A2" s="102"/>
+      <c r="B2" s="103"/>
+      <c r="C2" s="109"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="111"/>
       <c r="I2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="90">
+      <c r="J2" s="29">
         <v>1</v>
       </c>
-      <c r="L2" s="115" t="s">
-        <v>74</v>
+      <c r="L2" s="45" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74"/>
-      <c r="B3" s="75"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="84"/>
+      <c r="A3" s="102"/>
+      <c r="B3" s="103"/>
+      <c r="C3" s="109"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="111"/>
       <c r="I3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J3" s="91">
+      <c r="J3" s="30">
         <v>46251</v>
       </c>
-      <c r="L3" s="115" t="s">
-        <v>73</v>
+      <c r="L3" s="45" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="76"/>
-      <c r="B4" s="77"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="86"/>
-      <c r="E4" s="86"/>
-      <c r="F4" s="86"/>
-      <c r="G4" s="86"/>
-      <c r="H4" s="87"/>
+      <c r="A4" s="104"/>
+      <c r="B4" s="105"/>
+      <c r="C4" s="112"/>
+      <c r="D4" s="113"/>
+      <c r="E4" s="113"/>
+      <c r="F4" s="113"/>
+      <c r="G4" s="113"/>
+      <c r="H4" s="114"/>
       <c r="I4" s="1" t="s">
         <v>5</v>
       </c>
@@ -3168,10 +3128,10 @@
         <v>1680</v>
       </c>
       <c r="D6" s="17"/>
-      <c r="E6" s="78" t="s">
+      <c r="E6" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="78"/>
+      <c r="F6" s="28"/>
       <c r="G6" s="26">
         <f>+C6-4</f>
         <v>1676</v>
@@ -3188,525 +3148,525 @@
       <c r="E7" s="15"/>
       <c r="F7" s="15"/>
       <c r="H7" s="16"/>
-      <c r="I7" s="57"/>
-      <c r="J7" s="57"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
     </row>
     <row r="8" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="104" t="s">
+      <c r="A8" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="B8" s="104" t="s">
+      <c r="B8" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="105" t="s">
+      <c r="C8" s="115" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="105"/>
-      <c r="E8" s="105"/>
-      <c r="F8" s="104" t="s">
+      <c r="D8" s="115"/>
+      <c r="E8" s="115"/>
+      <c r="F8" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="H8" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="J8" s="38" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="43">
+        <v>1</v>
+      </c>
+      <c r="B9" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="90"/>
+      <c r="E9" s="90"/>
+      <c r="F9" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="43" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" s="43">
+        <v>7</v>
+      </c>
+      <c r="J9" s="43">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="46">
+        <v>2</v>
+      </c>
+      <c r="B10" s="46" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" s="90"/>
+      <c r="E10" s="90"/>
+      <c r="F10" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="G8" s="104" t="s">
-        <v>50</v>
-      </c>
-      <c r="H8" s="104" t="s">
-        <v>51</v>
-      </c>
-      <c r="I8" s="104" t="s">
-        <v>52</v>
-      </c>
-      <c r="J8" s="104" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="111">
-        <v>1</v>
-      </c>
-      <c r="B9" s="111" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D9" s="116"/>
-      <c r="E9" s="116"/>
-      <c r="F9" s="111" t="s">
+      <c r="G10" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="H10" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="I10" s="46">
+        <v>7</v>
+      </c>
+      <c r="J10" s="46">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="43">
+        <v>3</v>
+      </c>
+      <c r="B11" s="43" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11" s="90"/>
+      <c r="E11" s="90"/>
+      <c r="F11" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="G11" s="43" t="s">
+        <v>60</v>
+      </c>
+      <c r="H11" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="I11" s="43">
+        <v>7</v>
+      </c>
+      <c r="J11" s="43">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="43">
+        <v>4</v>
+      </c>
+      <c r="B12" s="46" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" s="90"/>
+      <c r="E12" s="90"/>
+      <c r="F12" s="43" t="s">
+        <v>69</v>
+      </c>
+      <c r="G12" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="H12" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="I12" s="46">
+        <v>28</v>
+      </c>
+      <c r="J12" s="46">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="46">
+        <v>5</v>
+      </c>
+      <c r="B13" s="43" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="90"/>
+      <c r="E13" s="90"/>
+      <c r="F13" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="43" t="s">
+        <v>60</v>
+      </c>
+      <c r="H13" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="I13" s="43">
+        <v>28</v>
+      </c>
+      <c r="J13" s="43">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="43">
+        <v>6</v>
+      </c>
+      <c r="B14" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14" s="90"/>
+      <c r="E14" s="90"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="I14" s="46">
+        <v>28</v>
+      </c>
+      <c r="J14" s="46">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="43">
+        <v>7</v>
+      </c>
+      <c r="B15" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D15" s="90"/>
+      <c r="E15" s="90"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="H15" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="I15" s="46">
+        <v>28</v>
+      </c>
+      <c r="J15" s="46">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="46">
+        <v>8</v>
+      </c>
+      <c r="B16" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" s="90"/>
+      <c r="E16" s="90"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="H16" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="I16" s="46">
+        <v>28</v>
+      </c>
+      <c r="J16" s="46">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="43">
+        <v>9</v>
+      </c>
+      <c r="B17" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D17" s="90"/>
+      <c r="E17" s="90"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="H17" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="I17" s="46">
+        <v>28</v>
+      </c>
+      <c r="J17" s="46">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="43">
         <v>10</v>
       </c>
-      <c r="G9" s="111" t="s">
+      <c r="B18" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18" s="90"/>
+      <c r="E18" s="90"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="H9" s="111" t="s">
+      <c r="H18" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="I9" s="111">
-        <v>7</v>
-      </c>
-      <c r="J9" s="111">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="117">
-        <v>2</v>
-      </c>
-      <c r="B10" s="117" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D10" s="116"/>
-      <c r="E10" s="116"/>
-      <c r="F10" s="111" t="s">
-        <v>68</v>
-      </c>
-      <c r="G10" s="117" t="s">
+      <c r="I18" s="46">
+        <v>28</v>
+      </c>
+      <c r="J18" s="46">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="46">
+        <v>11</v>
+      </c>
+      <c r="B19" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D19" s="90"/>
+      <c r="E19" s="90"/>
+      <c r="F19" s="43"/>
+      <c r="G19" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="H10" s="117" t="s">
+      <c r="H19" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="I10" s="117">
-        <v>7</v>
-      </c>
-      <c r="J10" s="117">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="111">
-        <v>3</v>
-      </c>
-      <c r="B11" s="111" t="s">
-        <v>56</v>
-      </c>
-      <c r="C11" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" s="116"/>
-      <c r="E11" s="116"/>
-      <c r="F11" s="111" t="s">
-        <v>69</v>
-      </c>
-      <c r="G11" s="111" t="s">
+      <c r="I19" s="46">
+        <v>28</v>
+      </c>
+      <c r="J19" s="46">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="43">
+        <v>12</v>
+      </c>
+      <c r="B20" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" s="90"/>
+      <c r="E20" s="90"/>
+      <c r="F20" s="43"/>
+      <c r="G20" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="H11" s="111" t="s">
+      <c r="H20" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="I11" s="111">
-        <v>7</v>
-      </c>
-      <c r="J11" s="111">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="111">
-        <v>4</v>
-      </c>
-      <c r="B12" s="117" t="s">
-        <v>57</v>
-      </c>
-      <c r="C12" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D12" s="116"/>
-      <c r="E12" s="116"/>
-      <c r="F12" s="111" t="s">
-        <v>70</v>
-      </c>
-      <c r="G12" s="117" t="s">
-        <v>60</v>
-      </c>
-      <c r="H12" s="117" t="s">
-        <v>61</v>
-      </c>
-      <c r="I12" s="117">
+      <c r="I20" s="46">
         <v>28</v>
       </c>
-      <c r="J12" s="117">
+      <c r="J20" s="46">
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="117">
-        <v>5</v>
-      </c>
-      <c r="B13" s="111" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D13" s="116"/>
-      <c r="E13" s="116"/>
-      <c r="F13" s="111" t="s">
-        <v>71</v>
-      </c>
-      <c r="G13" s="111" t="s">
-        <v>60</v>
-      </c>
-      <c r="H13" s="111" t="s">
-        <v>61</v>
-      </c>
-      <c r="I13" s="111">
-        <v>28</v>
-      </c>
-      <c r="J13" s="111">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="111">
-        <v>6</v>
-      </c>
-      <c r="B14" s="117" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D14" s="116"/>
-      <c r="E14" s="116"/>
-      <c r="F14" s="112"/>
-      <c r="G14" s="117" t="s">
-        <v>60</v>
-      </c>
-      <c r="H14" s="117" t="s">
-        <v>61</v>
-      </c>
-      <c r="I14" s="117">
-        <v>28</v>
-      </c>
-      <c r="J14" s="117">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="111">
-        <v>7</v>
-      </c>
-      <c r="B15" s="117" t="s">
-        <v>59</v>
-      </c>
-      <c r="C15" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D15" s="116"/>
-      <c r="E15" s="116"/>
-      <c r="F15" s="112"/>
-      <c r="G15" s="117" t="s">
-        <v>60</v>
-      </c>
-      <c r="H15" s="117" t="s">
-        <v>61</v>
-      </c>
-      <c r="I15" s="117">
-        <v>28</v>
-      </c>
-      <c r="J15" s="117">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="117">
-        <v>8</v>
-      </c>
-      <c r="B16" s="117" t="s">
-        <v>59</v>
-      </c>
-      <c r="C16" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D16" s="116"/>
-      <c r="E16" s="116"/>
-      <c r="F16" s="112"/>
-      <c r="G16" s="117" t="s">
-        <v>60</v>
-      </c>
-      <c r="H16" s="117" t="s">
-        <v>61</v>
-      </c>
-      <c r="I16" s="117">
-        <v>28</v>
-      </c>
-      <c r="J16" s="117">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="111">
-        <v>9</v>
-      </c>
-      <c r="B17" s="117" t="s">
-        <v>59</v>
-      </c>
-      <c r="C17" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D17" s="116"/>
-      <c r="E17" s="116"/>
-      <c r="F17" s="112"/>
-      <c r="G17" s="117" t="s">
-        <v>60</v>
-      </c>
-      <c r="H17" s="117" t="s">
-        <v>61</v>
-      </c>
-      <c r="I17" s="117">
-        <v>28</v>
-      </c>
-      <c r="J17" s="117">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="111">
-        <v>10</v>
-      </c>
-      <c r="B18" s="117" t="s">
-        <v>59</v>
-      </c>
-      <c r="C18" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D18" s="116"/>
-      <c r="E18" s="116"/>
-      <c r="F18" s="111"/>
-      <c r="G18" s="117" t="s">
-        <v>60</v>
-      </c>
-      <c r="H18" s="117" t="s">
-        <v>61</v>
-      </c>
-      <c r="I18" s="117">
-        <v>28</v>
-      </c>
-      <c r="J18" s="117">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="117">
-        <v>11</v>
-      </c>
-      <c r="B19" s="117" t="s">
-        <v>59</v>
-      </c>
-      <c r="C19" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D19" s="116"/>
-      <c r="E19" s="116"/>
-      <c r="F19" s="111"/>
-      <c r="G19" s="117" t="s">
-        <v>60</v>
-      </c>
-      <c r="H19" s="117" t="s">
-        <v>61</v>
-      </c>
-      <c r="I19" s="117">
-        <v>28</v>
-      </c>
-      <c r="J19" s="117">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="111">
-        <v>12</v>
-      </c>
-      <c r="B20" s="117" t="s">
-        <v>59</v>
-      </c>
-      <c r="C20" s="116" t="s">
-        <v>72</v>
-      </c>
-      <c r="D20" s="116"/>
-      <c r="E20" s="116"/>
-      <c r="F20" s="111"/>
-      <c r="G20" s="117" t="s">
-        <v>60</v>
-      </c>
-      <c r="H20" s="117" t="s">
-        <v>61</v>
-      </c>
-      <c r="I20" s="117">
-        <v>28</v>
-      </c>
-      <c r="J20" s="117">
-        <v>100</v>
-      </c>
-    </row>
     <row r="21" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="107"/>
-      <c r="B21" s="108"/>
-      <c r="C21" s="109"/>
-      <c r="D21" s="109"/>
-      <c r="E21" s="109"/>
-      <c r="F21" s="109"/>
-      <c r="G21" s="108"/>
-      <c r="H21" s="108"/>
-      <c r="I21" s="108"/>
-      <c r="J21" s="110"/>
+      <c r="A21" s="39"/>
+      <c r="B21" s="40"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40"/>
+      <c r="J21" s="42"/>
     </row>
     <row r="22" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="107"/>
-      <c r="B22" s="108"/>
-      <c r="C22" s="109"/>
-      <c r="D22" s="109"/>
-      <c r="E22" s="109"/>
-      <c r="F22" s="109"/>
-      <c r="G22" s="108"/>
-      <c r="H22" s="108"/>
-      <c r="I22" s="108"/>
-      <c r="J22" s="110"/>
+      <c r="A22" s="39"/>
+      <c r="B22" s="40"/>
+      <c r="C22" s="41"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="40"/>
+      <c r="J22" s="42"/>
     </row>
     <row r="23" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="71"/>
-      <c r="B23" s="71"/>
-      <c r="C23" s="71"/>
-      <c r="D23" s="71"/>
-      <c r="E23" s="71"/>
-      <c r="F23" s="71"/>
-      <c r="G23" s="71"/>
-      <c r="H23" s="71"/>
-      <c r="I23" s="71"/>
-      <c r="J23" s="71"/>
+      <c r="A23" s="15"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="15"/>
     </row>
     <row r="24" spans="1:10" ht="36.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="106" t="s">
+      <c r="A24" s="96" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="106"/>
-      <c r="C24" s="96">
+      <c r="B24" s="96"/>
+      <c r="C24" s="34">
         <v>46249</v>
       </c>
-      <c r="D24" s="106" t="s">
+      <c r="D24" s="96" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="106"/>
-      <c r="F24" s="113" t="str">
+      <c r="E24" s="96"/>
+      <c r="F24" s="97" t="str">
         <f>+G9</f>
         <v>2026/08/15</v>
       </c>
-      <c r="G24" s="114"/>
-      <c r="H24" s="106" t="s">
+      <c r="G24" s="98"/>
+      <c r="H24" s="96" t="s">
         <v>23</v>
       </c>
-      <c r="I24" s="106"/>
-      <c r="J24" s="96" t="str">
+      <c r="I24" s="96"/>
+      <c r="J24" s="34" t="str">
         <f>+F24</f>
         <v>2026/08/15</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="16.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="92"/>
-      <c r="B25" s="92"/>
-      <c r="C25" s="92"/>
-      <c r="D25" s="92"/>
-      <c r="E25" s="93"/>
-      <c r="F25" s="93"/>
-      <c r="G25" s="94"/>
-      <c r="H25" s="92"/>
-      <c r="I25" s="92"/>
-      <c r="J25" s="95"/>
+      <c r="A25" s="31"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="31"/>
+      <c r="J25" s="16"/>
     </row>
     <row r="26" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="103" t="s">
+      <c r="A26" s="95" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="103"/>
-      <c r="C26" s="98"/>
-      <c r="D26" s="98"/>
-      <c r="E26" s="98"/>
-      <c r="F26" s="98"/>
-      <c r="G26" s="98"/>
-      <c r="H26" s="98"/>
-      <c r="I26" s="98"/>
-      <c r="J26" s="98"/>
+      <c r="B26" s="95"/>
+      <c r="C26" s="36"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="36"/>
+      <c r="F26" s="36"/>
+      <c r="G26" s="36"/>
+      <c r="H26" s="36"/>
+      <c r="I26" s="36"/>
+      <c r="J26" s="36"/>
     </row>
     <row r="27" spans="1:10" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="98"/>
-      <c r="B27" s="98"/>
-      <c r="C27" s="98"/>
-      <c r="D27" s="98"/>
-      <c r="E27" s="98"/>
-      <c r="F27" s="98"/>
-      <c r="G27" s="98"/>
-      <c r="H27" s="98"/>
-      <c r="I27" s="98"/>
-      <c r="J27" s="98"/>
+      <c r="A27" s="36"/>
+      <c r="B27" s="36"/>
+      <c r="C27" s="36"/>
+      <c r="D27" s="36"/>
+      <c r="E27" s="36"/>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36"/>
+      <c r="I27" s="36"/>
+      <c r="J27" s="36"/>
     </row>
     <row r="28" spans="1:10" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="99"/>
-      <c r="B28" s="99"/>
-      <c r="C28" s="99"/>
-      <c r="D28" s="99"/>
-      <c r="E28" s="99"/>
-      <c r="F28" s="99"/>
-      <c r="G28" s="99"/>
-      <c r="H28" s="99"/>
-      <c r="I28" s="99"/>
-      <c r="J28" s="99"/>
+      <c r="A28" s="37"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="37"/>
+      <c r="I28" s="37"/>
+      <c r="J28" s="37"/>
     </row>
     <row r="29" spans="1:10" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="97"/>
-      <c r="B29" s="97"/>
-      <c r="C29" s="97"/>
-      <c r="D29" s="97"/>
-      <c r="E29" s="97"/>
-      <c r="F29" s="97"/>
-      <c r="G29" s="97"/>
-      <c r="H29" s="97"/>
-      <c r="I29" s="97"/>
-      <c r="J29" s="97"/>
+      <c r="A29" s="35"/>
+      <c r="B29" s="35"/>
+      <c r="C29" s="35"/>
+      <c r="D29" s="35"/>
+      <c r="E29" s="35"/>
+      <c r="F29" s="35"/>
+      <c r="G29" s="35"/>
+      <c r="H29" s="35"/>
+      <c r="I29" s="35"/>
+      <c r="J29" s="35"/>
     </row>
     <row r="30" spans="1:10" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="97"/>
-      <c r="B30" s="97"/>
-      <c r="C30" s="97"/>
-      <c r="D30" s="97"/>
-      <c r="E30" s="97"/>
-      <c r="F30" s="97"/>
-      <c r="G30" s="97"/>
-      <c r="H30" s="97"/>
-      <c r="I30" s="97"/>
-      <c r="J30" s="97"/>
+      <c r="A30" s="35"/>
+      <c r="B30" s="35"/>
+      <c r="C30" s="35"/>
+      <c r="D30" s="35"/>
+      <c r="E30" s="35"/>
+      <c r="F30" s="35"/>
+      <c r="G30" s="35"/>
+      <c r="H30" s="35"/>
+      <c r="I30" s="35"/>
+      <c r="J30" s="35"/>
     </row>
     <row r="31" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="97"/>
-      <c r="B31" s="97"/>
-      <c r="C31" s="97"/>
-      <c r="D31" s="97"/>
-      <c r="E31" s="97"/>
-      <c r="F31" s="97"/>
-      <c r="G31" s="97"/>
-      <c r="H31" s="97"/>
-      <c r="I31" s="97"/>
-      <c r="J31" s="97"/>
+      <c r="A31" s="35"/>
+      <c r="B31" s="35"/>
+      <c r="C31" s="35"/>
+      <c r="D31" s="35"/>
+      <c r="E31" s="35"/>
+      <c r="F31" s="35"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="35"/>
+      <c r="I31" s="35"/>
+      <c r="J31" s="35"/>
     </row>
     <row r="32" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="1:10" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="100" t="s">
+      <c r="A33" s="91" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="101"/>
-      <c r="C33" s="48" t="s">
-        <v>66</v>
-      </c>
-      <c r="D33" s="48"/>
-      <c r="E33" s="48"/>
-      <c r="F33" s="100" t="s">
-        <v>64</v>
-      </c>
-      <c r="G33" s="102"/>
-      <c r="H33" s="101"/>
-      <c r="I33" s="88"/>
-      <c r="J33" s="89"/>
+      <c r="B33" s="92"/>
+      <c r="C33" s="49" t="s">
+        <v>65</v>
+      </c>
+      <c r="D33" s="49"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="91" t="s">
+        <v>74</v>
+      </c>
+      <c r="G33" s="99"/>
+      <c r="H33" s="92"/>
+      <c r="I33" s="93"/>
+      <c r="J33" s="94"/>
     </row>
     <row r="40" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="41" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -3714,12 +3674,16 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="A1:B4"/>
+    <mergeCell ref="C1:H4"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="C9:E9"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="C33:E33"/>
     <mergeCell ref="I33:J33"/>
@@ -3728,17 +3692,13 @@
     <mergeCell ref="H24:I24"/>
     <mergeCell ref="F24:G24"/>
     <mergeCell ref="F33:H33"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="A1:B4"/>
-    <mergeCell ref="C1:H4"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C20:E20"/>
     <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C18:E18"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.78740157480314965" bottom="0.39370078740157483" header="0" footer="0"/>
@@ -3772,16 +3732,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="48"/>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="58" t="s">
+      <c r="A1" s="49"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
       <c r="I1" s="1" t="s">
         <v>1</v>
       </c>
@@ -3790,14 +3750,14 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
+      <c r="A2" s="49"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
       <c r="I2" s="1" t="s">
         <v>3</v>
       </c>
@@ -3806,14 +3766,14 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="48"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
+      <c r="A3" s="49"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
       <c r="I3" s="1" t="s">
         <v>4</v>
       </c>
@@ -3822,14 +3782,14 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="48"/>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
+      <c r="A4" s="49"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
       <c r="I4" s="1" t="s">
         <v>5</v>
       </c>
@@ -3854,10 +3814,10 @@
       <c r="A6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="56">
+      <c r="B6" s="47">
         <v>875</v>
       </c>
-      <c r="C6" s="56"/>
+      <c r="C6" s="47"/>
       <c r="D6" s="16"/>
       <c r="E6" s="15"/>
       <c r="F6" s="15" t="s">
@@ -3883,10 +3843,10 @@
       <c r="F7" s="15"/>
       <c r="G7" s="15"/>
       <c r="H7" s="16"/>
-      <c r="I7" s="57" t="s">
+      <c r="I7" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="57"/>
+      <c r="J7" s="48"/>
     </row>
     <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14"/>
@@ -3904,18 +3864,18 @@
       <c r="A9" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="77" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28" t="s">
+      <c r="C9" s="77"/>
+      <c r="D9" s="77"/>
+      <c r="E9" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
+      <c r="F9" s="77"/>
+      <c r="G9" s="77"/>
+      <c r="H9" s="77"/>
+      <c r="I9" s="77"/>
       <c r="J9" s="13" t="s">
         <v>15</v>
       </c>
@@ -3924,315 +3884,315 @@
       <c r="A10" s="12">
         <v>1</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="73" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="64" t="s">
+      <c r="C10" s="74"/>
+      <c r="D10" s="74"/>
+      <c r="E10" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="68"/>
-      <c r="G10" s="68"/>
-      <c r="H10" s="68"/>
-      <c r="I10" s="69"/>
+      <c r="F10" s="81"/>
+      <c r="G10" s="81"/>
+      <c r="H10" s="81"/>
+      <c r="I10" s="82"/>
       <c r="J10" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
-      <c r="B11" s="41"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="31" t="s">
+      <c r="B11" s="54"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="55"/>
+      <c r="E11" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="33"/>
+      <c r="F11" s="52"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="52"/>
+      <c r="I11" s="53"/>
       <c r="J11" s="12">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12"/>
-      <c r="B12" s="36"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="64" t="s">
+      <c r="B12" s="78"/>
+      <c r="C12" s="79"/>
+      <c r="D12" s="79"/>
+      <c r="E12" s="83" t="s">
         <v>35</v>
       </c>
-      <c r="F12" s="65"/>
-      <c r="G12" s="65"/>
-      <c r="H12" s="65"/>
-      <c r="I12" s="66"/>
+      <c r="F12" s="84"/>
+      <c r="G12" s="84"/>
+      <c r="H12" s="84"/>
+      <c r="I12" s="85"/>
       <c r="J12" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12"/>
-      <c r="B13" s="48"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="31" t="s">
+      <c r="B13" s="49"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="33"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="52"/>
+      <c r="I13" s="53"/>
       <c r="J13" s="12">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12"/>
-      <c r="B14" s="34"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="45" t="s">
+      <c r="B14" s="73"/>
+      <c r="C14" s="74"/>
+      <c r="D14" s="74"/>
+      <c r="E14" s="72" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="39"/>
-      <c r="I14" s="40"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="61"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="62"/>
       <c r="J14" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="70" t="s">
+      <c r="B15" s="73"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="80" t="s">
         <v>38</v>
       </c>
-      <c r="F15" s="68"/>
-      <c r="G15" s="68"/>
-      <c r="H15" s="68"/>
-      <c r="I15" s="69"/>
+      <c r="F15" s="81"/>
+      <c r="G15" s="81"/>
+      <c r="H15" s="81"/>
+      <c r="I15" s="82"/>
       <c r="J15" s="12">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="12"/>
-      <c r="B16" s="34"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="61" t="s">
+      <c r="B16" s="73"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="86" t="s">
         <v>39</v>
       </c>
-      <c r="F16" s="62"/>
-      <c r="G16" s="62"/>
-      <c r="H16" s="62"/>
-      <c r="I16" s="63"/>
+      <c r="F16" s="87"/>
+      <c r="G16" s="87"/>
+      <c r="H16" s="87"/>
+      <c r="I16" s="88"/>
       <c r="J16" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12"/>
-      <c r="B17" s="45"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="64" t="s">
+      <c r="B17" s="72"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="62"/>
+      <c r="E17" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="F17" s="65"/>
-      <c r="G17" s="65"/>
-      <c r="H17" s="65"/>
-      <c r="I17" s="66"/>
+      <c r="F17" s="84"/>
+      <c r="G17" s="84"/>
+      <c r="H17" s="84"/>
+      <c r="I17" s="85"/>
       <c r="J17" s="12">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12"/>
-      <c r="B18" s="34"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="67" t="s">
+      <c r="B18" s="73"/>
+      <c r="C18" s="74"/>
+      <c r="D18" s="74"/>
+      <c r="E18" s="89" t="s">
         <v>48</v>
       </c>
-      <c r="F18" s="68"/>
-      <c r="G18" s="68"/>
-      <c r="H18" s="68"/>
-      <c r="I18" s="69"/>
+      <c r="F18" s="81"/>
+      <c r="G18" s="81"/>
+      <c r="H18" s="81"/>
+      <c r="I18" s="82"/>
       <c r="J18" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12"/>
-      <c r="B19" s="29"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="32"/>
-      <c r="I19" s="33"/>
+      <c r="B19" s="58"/>
+      <c r="C19" s="59"/>
+      <c r="D19" s="59"/>
+      <c r="E19" s="51"/>
+      <c r="F19" s="52"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="52"/>
+      <c r="I19" s="53"/>
       <c r="J19" s="12"/>
     </row>
     <row r="20" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="12"/>
-      <c r="B20" s="41"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="64"/>
-      <c r="F20" s="65"/>
-      <c r="G20" s="65"/>
-      <c r="H20" s="65"/>
-      <c r="I20" s="66"/>
+      <c r="B20" s="54"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="83"/>
+      <c r="F20" s="84"/>
+      <c r="G20" s="84"/>
+      <c r="H20" s="84"/>
+      <c r="I20" s="85"/>
       <c r="J20" s="12"/>
     </row>
     <row r="21" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="32"/>
-      <c r="I21" s="33"/>
+      <c r="B21" s="58"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="51"/>
+      <c r="F21" s="52"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="52"/>
+      <c r="I21" s="53"/>
       <c r="J21" s="12"/>
     </row>
     <row r="22" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12"/>
-      <c r="B22" s="34"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="61"/>
-      <c r="F22" s="62"/>
-      <c r="G22" s="62"/>
-      <c r="H22" s="62"/>
-      <c r="I22" s="63"/>
+      <c r="B22" s="73"/>
+      <c r="C22" s="74"/>
+      <c r="D22" s="74"/>
+      <c r="E22" s="86"/>
+      <c r="F22" s="87"/>
+      <c r="G22" s="87"/>
+      <c r="H22" s="87"/>
+      <c r="I22" s="88"/>
       <c r="J22" s="12"/>
     </row>
     <row r="23" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="12"/>
-      <c r="B23" s="41"/>
-      <c r="C23" s="42"/>
-      <c r="D23" s="42"/>
-      <c r="E23" s="64"/>
-      <c r="F23" s="65"/>
-      <c r="G23" s="65"/>
-      <c r="H23" s="65"/>
-      <c r="I23" s="66"/>
+      <c r="B23" s="54"/>
+      <c r="C23" s="55"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="83"/>
+      <c r="F23" s="84"/>
+      <c r="G23" s="84"/>
+      <c r="H23" s="84"/>
+      <c r="I23" s="85"/>
       <c r="J23" s="12"/>
     </row>
     <row r="24" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
-      <c r="B24" s="48"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="33"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="51"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="52"/>
+      <c r="H24" s="52"/>
+      <c r="I24" s="53"/>
       <c r="J24" s="12"/>
     </row>
     <row r="25" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12"/>
-      <c r="B25" s="41"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="48"/>
-      <c r="H25" s="48"/>
-      <c r="I25" s="48"/>
+      <c r="B25" s="54"/>
+      <c r="C25" s="55"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="57"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="49"/>
       <c r="J25" s="12"/>
     </row>
     <row r="26" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="12"/>
-      <c r="B26" s="41"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="33"/>
+      <c r="B26" s="54"/>
+      <c r="C26" s="55"/>
+      <c r="D26" s="55"/>
+      <c r="E26" s="56"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="52"/>
+      <c r="I26" s="53"/>
       <c r="J26" s="12"/>
     </row>
     <row r="27" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="12"/>
-      <c r="B27" s="48"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
-      <c r="I27" s="48"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="49"/>
+      <c r="D27" s="49"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="49"/>
+      <c r="H27" s="49"/>
+      <c r="I27" s="49"/>
       <c r="J27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="12"/>
-      <c r="B28" s="48"/>
-      <c r="C28" s="48"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="33"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="52"/>
+      <c r="H28" s="52"/>
+      <c r="I28" s="53"/>
       <c r="J28" s="12"/>
     </row>
     <row r="29" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="12"/>
-      <c r="B29" s="48"/>
-      <c r="C29" s="48"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="40"/>
+      <c r="B29" s="49"/>
+      <c r="C29" s="49"/>
+      <c r="D29" s="49"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="61"/>
+      <c r="G29" s="61"/>
+      <c r="H29" s="61"/>
+      <c r="I29" s="62"/>
       <c r="J29" s="22"/>
     </row>
     <row r="30" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="12"/>
-      <c r="B30" s="48"/>
-      <c r="C30" s="48"/>
-      <c r="D30" s="48"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
-      <c r="I30" s="33"/>
+      <c r="B30" s="49"/>
+      <c r="C30" s="49"/>
+      <c r="D30" s="49"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="52"/>
+      <c r="H30" s="52"/>
+      <c r="I30" s="53"/>
       <c r="J30" s="12"/>
     </row>
     <row r="31" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="12"/>
-      <c r="B31" s="48"/>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="48"/>
-      <c r="H31" s="48"/>
-      <c r="I31" s="48"/>
+      <c r="B31" s="49"/>
+      <c r="C31" s="49"/>
+      <c r="D31" s="49"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="49"/>
+      <c r="G31" s="49"/>
+      <c r="H31" s="49"/>
+      <c r="I31" s="49"/>
       <c r="J31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="55" t="s">
+      <c r="A32" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="B32" s="55"/>
-      <c r="C32" s="51">
+      <c r="B32" s="64"/>
+      <c r="C32" s="69">
         <v>45566</v>
       </c>
-      <c r="D32" s="52"/>
+      <c r="D32" s="70"/>
       <c r="E32" s="5" t="s">
         <v>19</v>
       </c>
@@ -4249,15 +4209,15 @@
       <c r="J32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="55" t="s">
+      <c r="A33" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="55"/>
-      <c r="C33" s="53">
+      <c r="B33" s="64"/>
+      <c r="C33" s="71">
         <f>+F33-F32+1</f>
         <v>4</v>
       </c>
-      <c r="D33" s="53"/>
+      <c r="D33" s="71"/>
       <c r="E33" s="5" t="s">
         <v>23</v>
       </c>
@@ -4274,88 +4234,88 @@
       <c r="J33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="54" t="s">
+      <c r="A34" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B34" s="54"/>
-      <c r="C34" s="54"/>
-      <c r="D34" s="54"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="54"/>
-      <c r="G34" s="54"/>
-      <c r="H34" s="54"/>
-      <c r="I34" s="54"/>
-      <c r="J34" s="54"/>
+      <c r="B34" s="63"/>
+      <c r="C34" s="63"/>
+      <c r="D34" s="63"/>
+      <c r="E34" s="63"/>
+      <c r="F34" s="63"/>
+      <c r="G34" s="63"/>
+      <c r="H34" s="63"/>
+      <c r="I34" s="63"/>
+      <c r="J34" s="63"/>
     </row>
     <row r="35" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="46" t="s">
+      <c r="A35" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="B35" s="46"/>
-      <c r="C35" s="46"/>
-      <c r="D35" s="46"/>
-      <c r="E35" s="46"/>
-      <c r="F35" s="46"/>
-      <c r="G35" s="46"/>
-      <c r="H35" s="46"/>
-      <c r="I35" s="46"/>
-      <c r="J35" s="46"/>
+      <c r="B35" s="65"/>
+      <c r="C35" s="65"/>
+      <c r="D35" s="65"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="65"/>
+      <c r="G35" s="65"/>
+      <c r="H35" s="65"/>
+      <c r="I35" s="65"/>
+      <c r="J35" s="65"/>
     </row>
     <row r="36" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="46"/>
-      <c r="B36" s="46"/>
-      <c r="C36" s="46"/>
-      <c r="D36" s="46"/>
-      <c r="E36" s="46"/>
-      <c r="F36" s="46"/>
-      <c r="G36" s="46"/>
-      <c r="H36" s="46"/>
-      <c r="I36" s="46"/>
-      <c r="J36" s="46"/>
+      <c r="A36" s="65"/>
+      <c r="B36" s="65"/>
+      <c r="C36" s="65"/>
+      <c r="D36" s="65"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="65"/>
+      <c r="G36" s="65"/>
+      <c r="H36" s="65"/>
+      <c r="I36" s="65"/>
+      <c r="J36" s="65"/>
     </row>
     <row r="37" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="46"/>
-      <c r="B37" s="46"/>
-      <c r="C37" s="46"/>
-      <c r="D37" s="46"/>
-      <c r="E37" s="46"/>
-      <c r="F37" s="46"/>
-      <c r="G37" s="46"/>
-      <c r="H37" s="46"/>
-      <c r="I37" s="46"/>
-      <c r="J37" s="46"/>
+      <c r="A37" s="65"/>
+      <c r="B37" s="65"/>
+      <c r="C37" s="65"/>
+      <c r="D37" s="65"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="65"/>
+      <c r="H37" s="65"/>
+      <c r="I37" s="65"/>
+      <c r="J37" s="65"/>
     </row>
     <row r="38" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="46"/>
-      <c r="B38" s="46"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="46"/>
-      <c r="F38" s="46"/>
-      <c r="G38" s="46"/>
-      <c r="H38" s="46"/>
-      <c r="I38" s="46"/>
-      <c r="J38" s="46"/>
+      <c r="A38" s="65"/>
+      <c r="B38" s="65"/>
+      <c r="C38" s="65"/>
+      <c r="D38" s="65"/>
+      <c r="E38" s="65"/>
+      <c r="F38" s="65"/>
+      <c r="G38" s="65"/>
+      <c r="H38" s="65"/>
+      <c r="I38" s="65"/>
+      <c r="J38" s="65"/>
     </row>
     <row r="39" spans="1:10" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="49" t="s">
+      <c r="A39" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="B39" s="50"/>
-      <c r="C39" s="45" t="s">
+      <c r="B39" s="68"/>
+      <c r="C39" s="72" t="s">
         <v>29</v>
       </c>
-      <c r="D39" s="39"/>
-      <c r="E39" s="39"/>
-      <c r="F39" s="40"/>
+      <c r="D39" s="61"/>
+      <c r="E39" s="61"/>
+      <c r="F39" s="62"/>
       <c r="G39" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="H39" s="47" t="s">
+      <c r="H39" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="I39" s="48"/>
-      <c r="J39" s="48"/>
+      <c r="I39" s="49"/>
+      <c r="J39" s="49"/>
     </row>
     <row r="46" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4363,48 +4323,11 @@
     </row>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="A1:D4"/>
-    <mergeCell ref="E1:H4"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="E9:I9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:I10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="E11:I11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="E12:I12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:I13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="E14:I14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="E15:I15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="E16:I16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E18:I18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E19:I19"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="E20:I20"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E21:I21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="E22:I22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="A34:J34"/>
+    <mergeCell ref="A35:J38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="C39:F39"/>
+    <mergeCell ref="H39:J39"/>
     <mergeCell ref="C33:D33"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="E28:I28"/>
@@ -4417,11 +4340,48 @@
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="C32:D32"/>
     <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:J34"/>
-    <mergeCell ref="A35:J38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C39:F39"/>
-    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E22:I22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E19:I19"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="E20:I20"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E21:I21"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="E16:I16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:I18"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:I13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E14:I14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E15:I15"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:I10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="E11:I11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="E12:I12"/>
+    <mergeCell ref="A1:D4"/>
+    <mergeCell ref="E1:H4"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="E9:I9"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.59055118110236227" right="0.39370078740157483" top="0.78740157480314965" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>

<commit_message>
feat(ot): wrap text in F33:H33, auto-evaluate EMITIDO status, map fin_programado to fecha_estimada_culminacion, and remove silent background OT sync
</commit_message>
<xml_diff>
--- a/app/templates/OT/OT-CONCRETO/OT-0000-Geofal.xlsx
+++ b/app/templates/OT/OT-CONCRETO/OT-0000-Geofal.xlsx
@@ -366,7 +366,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="147">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -773,6 +773,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3617,13 +3623,14 @@
       </c>
       <c r="D33" s="128" t="n"/>
       <c r="E33" s="124" t="n"/>
-      <c r="F33" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OT DESIGADA A:                                                                  </t>
-        </is>
-      </c>
-      <c r="G33" s="128" t="n"/>
-      <c r="H33" s="124" t="n"/>
+      <c r="F33" s="70" t="inlineStr">
+        <is>
+          <t>OT DESIGNADA A:
+(Colocar el nombre de los técnicos)</t>
+        </is>
+      </c>
+      <c r="G33" s="145" t="n"/>
+      <c r="H33" s="146" t="n"/>
       <c r="I33" s="49" t="n"/>
       <c r="J33" s="124" t="n"/>
     </row>

</xml_diff>